<commit_message>
Signed-off-by: Student George Tolkachov (TL_KCOMP_B_Y3) <t00262291@mymtu.ie>
</commit_message>
<xml_diff>
--- a/Assignment1_HT.xlsx
+++ b/Assignment1_HT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\StudentGeorgeTolkach\Desktop\CG_2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8853DD4D-91B6-48EE-A1B8-9FF2A7725961}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6503E64C-5135-495F-8D22-6E2E2361E1E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -559,44 +559,44 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -622,23 +622,23 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>593910</xdr:colOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>89645</xdr:rowOff>
+      <xdr:rowOff>1</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>1748118</xdr:colOff>
+      <xdr:colOff>1810537</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>5129563</xdr:rowOff>
+      <xdr:rowOff>5154707</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="Picture 4">
+        <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DB41D6B9-7C54-DF9E-E2BF-CA2760AA4C93}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C970CF89-38B9-269D-4D73-EC0C4B2ECF8F}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -646,17 +646,16 @@
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
-      <xdr:blipFill rotWithShape="1">
+      <xdr:blipFill>
         <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:srcRect l="-3951" r="39737"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1804145" y="403410"/>
-          <a:ext cx="1759326" cy="5039918"/>
+          <a:off x="1815353" y="313766"/>
+          <a:ext cx="1810537" cy="5154706"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -668,22 +667,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>1692088</xdr:colOff>
+      <xdr:colOff>1692089</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>112057</xdr:rowOff>
+      <xdr:rowOff>11208</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>1255058</xdr:colOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>42761</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>1613647</xdr:rowOff>
+      <xdr:rowOff>4011706</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="6" name="Picture 5">
+        <xdr:cNvPr id="3" name="Picture 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{62A65F92-1343-606E-0687-2E28E751221B}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A8422326-FB7B-3B65-C523-5098A4492CB5}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -691,17 +690,16 @@
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
-      <xdr:blipFill rotWithShape="1">
+      <xdr:blipFill>
         <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
-        <a:srcRect t="78986" r="19608"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3507441" y="425822"/>
-          <a:ext cx="2073088" cy="1501590"/>
+          <a:off x="3507442" y="324973"/>
+          <a:ext cx="2127054" cy="4000498"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -713,22 +711,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>324970</xdr:colOff>
+      <xdr:colOff>739588</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>100853</xdr:rowOff>
+      <xdr:rowOff>156883</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>863277</xdr:colOff>
+      <xdr:colOff>782526</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>1558381</xdr:rowOff>
+      <xdr:rowOff>1614411</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="7" name="Picture 6">
+        <xdr:cNvPr id="4" name="Picture 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{612A8402-1A1D-7BBC-887A-8945B35FC80A}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DFAB4443-2214-0E6E-7AEC-C1F5FFC04853}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -744,8 +742,363 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2140323" y="5916706"/>
-          <a:ext cx="3048425" cy="1457528"/>
+          <a:off x="2554941" y="5972736"/>
+          <a:ext cx="2553056" cy="1457528"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>201708</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1860176</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>5188325</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="Picture 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{62C6102E-A7A4-E9E4-0350-9E4643359D55}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:srcRect r="9564"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1815354" y="7933767"/>
+          <a:ext cx="1860175" cy="5221940"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1860177</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>224120</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>1232647</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>4244730</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="Picture 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D6D012E3-A423-E292-D6DF-47BDA28331F6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:srcRect r="14647"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3675530" y="7956179"/>
+          <a:ext cx="1882588" cy="4255933"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>627530</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>11209</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>896470</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>1165412</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="10" name="Picture 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{84E6FF8B-CF2C-4C4E-7C78-9D6EAC438BB6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2442883" y="13491885"/>
+          <a:ext cx="2779058" cy="1154203"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>78442</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>89647</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1793803</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>4971280</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="11" name="Picture 10">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E8BC7430-4BAC-25E0-ADEF-7175118509BE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1893795" y="15060706"/>
+          <a:ext cx="1715361" cy="4881633"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1792943</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>100853</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>38763</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>3944471</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="12" name="Picture 11">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F7868C7E-6AA6-DDCB-922C-64B8A9885F0F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3608296" y="15071912"/>
+          <a:ext cx="2022202" cy="3843618"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>526679</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>145676</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>694764</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>16753</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="13" name="Picture 12">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2C6B44D0-51E2-7037-C21A-32B29836F060}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2342032" y="20473147"/>
+          <a:ext cx="2678203" cy="1395077"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>33620</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>78441</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1843231</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>22411</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="14" name="Picture 13">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{672C0E0C-CDFA-94BA-1EE0-8DA9D3C21A4D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1848973" y="22243676"/>
+          <a:ext cx="1809611" cy="5143500"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1882593</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>78441</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>1242649</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>4258236</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="15" name="Picture 14">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{31CAA55F-30E4-A37E-E396-8137F17D9156}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11"/>
+        <a:srcRect r="11346"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3697946" y="22243676"/>
+          <a:ext cx="1870174" cy="4179795"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1057,24 +1410,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="38" t="s">
+      <c r="A1" s="49" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="38"/>
-      <c r="C1" s="38"/>
-      <c r="D1" s="38"/>
-      <c r="E1" s="38"/>
-      <c r="F1" s="38"/>
+      <c r="B1" s="49"/>
+      <c r="C1" s="49"/>
+      <c r="D1" s="49"/>
+      <c r="E1" s="49"/>
+      <c r="F1" s="49"/>
     </row>
     <row r="2" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="39" t="s">
+      <c r="A2" s="50" t="s">
         <v>36</v>
       </c>
-      <c r="B2" s="39"/>
-      <c r="C2" s="39"/>
-      <c r="D2" s="39"/>
-      <c r="E2" s="39"/>
-      <c r="F2" s="39"/>
+      <c r="B2" s="50"/>
+      <c r="C2" s="50"/>
+      <c r="D2" s="50"/>
+      <c r="E2" s="50"/>
+      <c r="F2" s="50"/>
     </row>
     <row r="3" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
@@ -1086,7 +1439,7 @@
         <v>22</v>
       </c>
       <c r="C4" s="26">
-        <v>366252</v>
+        <v>262291</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -1098,7 +1451,7 @@
       </c>
       <c r="C6" s="27">
         <f>MOD(C4,100)-50</f>
-        <v>2</v>
+        <v>41</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="12.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -1110,22 +1463,22 @@
       </c>
       <c r="C7" s="28">
         <f>C21/$G$21</f>
-        <v>0.99076429675591937</v>
+        <v>0.98019605881960692</v>
       </c>
       <c r="D7" s="27">
         <f t="shared" ref="D7:E7" si="0">D21/$G$21</f>
-        <v>-9.5880415815088965E-2</v>
+        <v>-0.140028008402801</v>
       </c>
       <c r="E7" s="29">
         <f t="shared" si="0"/>
-        <v>-9.5880415815088965E-2</v>
+        <v>-0.140028008402801</v>
       </c>
       <c r="F7" s="30" t="s">
         <v>37</v>
       </c>
       <c r="G7" s="33">
         <f>C21</f>
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="H7" s="25">
         <f t="shared" ref="H7:I7" si="1">D21</f>
@@ -1148,11 +1501,11 @@
       </c>
       <c r="C8" s="28">
         <f>C22</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D8" s="27">
         <f t="shared" ref="D8:E8" si="2">D22</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E8" s="29">
         <f t="shared" si="2"/>
@@ -1168,11 +1521,11 @@
       </c>
       <c r="C9" s="28">
         <f>C23</f>
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="D9" s="27">
         <f t="shared" ref="D9:E9" si="3">D23</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E9" s="29">
         <f t="shared" si="3"/>
@@ -1191,7 +1544,7 @@
       </c>
       <c r="C11" s="28">
         <f>C25</f>
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="D11" s="27">
         <f t="shared" ref="D11:E11" si="4">D25</f>
@@ -1213,7 +1566,7 @@
       </c>
       <c r="D12" s="36">
         <f t="shared" ref="D12:E12" si="5">D26</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E12" s="29">
         <f t="shared" si="5"/>
@@ -1230,15 +1583,15 @@
       </c>
       <c r="C13" s="28">
         <f>C27/$G$27</f>
-        <v>-6.4084133611200148E-2</v>
+        <v>-9.3864650892786422E-2</v>
       </c>
       <c r="D13" s="27">
         <f t="shared" ref="D13:E13" si="6">D27/$G$27</f>
-        <v>-9.6126200416800214E-2</v>
+        <v>-0.14079697633917962</v>
       </c>
       <c r="E13" s="29">
         <f t="shared" si="6"/>
-        <v>0.99330407097360229</v>
+        <v>0.98557883437425742</v>
       </c>
       <c r="F13" s="30" t="s">
         <v>32</v>
@@ -1253,7 +1606,7 @@
       </c>
       <c r="I13" s="34">
         <f t="shared" si="7"/>
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="J13" s="35" t="s">
         <v>39</v>
@@ -1297,7 +1650,7 @@
     <row r="21" spans="1:7" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C21" s="31">
         <f>INT((C4/10000))-5</f>
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="D21" s="31">
         <f>MOD(INT((C4/100)),10)-5</f>
@@ -1309,17 +1662,17 @@
       </c>
       <c r="G21" s="25">
         <f>SQRT(C21*C21+D21*D21+E21*E21)</f>
-        <v>31.28897569432403</v>
+        <v>21.42428528562855</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C22" s="32">
         <f>MOD(INT((C4/10000)),6) + 1</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D22" s="32">
         <f>MOD(MOD(INT((C4/1000)),10),6) +1</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E22" s="32">
         <f>MOD(MOD(INT((C4/100)),10),6) +1</f>
@@ -1327,17 +1680,17 @@
       </c>
       <c r="G22" s="25">
         <f t="shared" ref="G22:G27" si="8">SQRT(C22*C22+D22*D22+E22*E22)</f>
-        <v>3.3166247903553998</v>
+        <v>5.196152422706632</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C23" s="27">
         <f>MOD(C4,10)-5</f>
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="D23" s="27">
         <f>MOD(INT((C4/10)),10)-5</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E23" s="27">
         <f>MOD(INT((C4/100)),10)-4</f>
@@ -1345,7 +1698,7 @@
       </c>
       <c r="G23" s="25">
         <f t="shared" si="8"/>
-        <v>3.6055512754639891</v>
+        <v>6</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1357,7 +1710,7 @@
     <row r="25" spans="1:7" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C25" s="27">
         <f>2+C21</f>
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="D25" s="27">
         <f>3+D21</f>
@@ -1369,7 +1722,7 @@
       </c>
       <c r="G25" s="25">
         <f t="shared" si="8"/>
-        <v>57.428216061444921</v>
+        <v>52.32590180780452</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
@@ -1379,7 +1732,7 @@
       </c>
       <c r="D26" s="31">
         <f>C22</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E26" s="31">
         <f>E22</f>
@@ -1387,7 +1740,7 @@
       </c>
       <c r="G26" s="25">
         <f t="shared" si="8"/>
-        <v>4.358898943540674</v>
+        <v>5.196152422706632</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
@@ -1402,11 +1755,11 @@
       </c>
       <c r="E27" s="31">
         <f>C21</f>
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="G27" s="25">
         <f t="shared" si="8"/>
-        <v>31.208973068654469</v>
+        <v>21.307275752662516</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -1456,10 +1809,10 @@
     </row>
     <row r="2" spans="3:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C2" s="4"/>
-      <c r="D2" s="42" t="s">
+      <c r="D2" s="46" t="s">
         <v>35</v>
       </c>
-      <c r="E2" s="43"/>
+      <c r="E2" s="47"/>
       <c r="F2" s="7"/>
       <c r="G2" s="3"/>
       <c r="H2" s="3"/>
@@ -1470,8 +1823,8 @@
     </row>
     <row r="3" spans="3:13" ht="408.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C3" s="4"/>
-      <c r="D3" s="40"/>
-      <c r="E3" s="41"/>
+      <c r="D3" s="38"/>
+      <c r="E3" s="40"/>
       <c r="F3" s="5"/>
       <c r="G3" s="10"/>
       <c r="H3" s="6"/>
@@ -1491,10 +1844,10 @@
     </row>
     <row r="5" spans="3:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C5" s="4"/>
-      <c r="D5" s="42" t="s">
+      <c r="D5" s="46" t="s">
         <v>13</v>
       </c>
-      <c r="E5" s="43"/>
+      <c r="E5" s="47"/>
       <c r="F5" s="7"/>
       <c r="H5" s="14"/>
       <c r="I5" s="11"/>
@@ -1503,8 +1856,8 @@
     </row>
     <row r="6" spans="3:13" ht="138.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C6" s="4"/>
-      <c r="D6" s="40"/>
-      <c r="E6" s="41"/>
+      <c r="D6" s="38"/>
+      <c r="E6" s="40"/>
       <c r="F6" s="15"/>
       <c r="G6" s="11"/>
       <c r="H6" s="14"/>
@@ -1524,10 +1877,10 @@
     </row>
     <row r="8" spans="3:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C8" s="4"/>
-      <c r="D8" s="42" t="s">
+      <c r="D8" s="46" t="s">
         <v>30</v>
       </c>
-      <c r="E8" s="43"/>
+      <c r="E8" s="47"/>
       <c r="F8" s="16"/>
       <c r="G8" s="11"/>
       <c r="H8" s="14"/>
@@ -1537,8 +1890,8 @@
     </row>
     <row r="9" spans="3:13" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C9" s="4"/>
-      <c r="D9" s="40"/>
-      <c r="E9" s="41"/>
+      <c r="D9" s="38"/>
+      <c r="E9" s="40"/>
       <c r="F9" s="16"/>
       <c r="G9" s="11"/>
       <c r="H9" s="14"/>
@@ -1558,10 +1911,10 @@
     </row>
     <row r="11" spans="3:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C11" s="4"/>
-      <c r="D11" s="42" t="s">
+      <c r="D11" s="46" t="s">
         <v>4</v>
       </c>
-      <c r="E11" s="43"/>
+      <c r="E11" s="47"/>
       <c r="F11" s="17"/>
       <c r="G11" s="18"/>
       <c r="H11" s="44" t="s">
@@ -1574,12 +1927,12 @@
     </row>
     <row r="12" spans="3:13" ht="93" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C12" s="4"/>
-      <c r="D12" s="40"/>
-      <c r="E12" s="41"/>
+      <c r="D12" s="38"/>
+      <c r="E12" s="40"/>
       <c r="F12" s="15"/>
       <c r="G12" s="15"/>
-      <c r="H12" s="40"/>
-      <c r="I12" s="41"/>
+      <c r="H12" s="38"/>
+      <c r="I12" s="40"/>
       <c r="J12" s="15"/>
       <c r="K12" s="11"/>
       <c r="L12" s="14"/>
@@ -1599,10 +1952,10 @@
     </row>
     <row r="14" spans="3:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C14" s="4"/>
-      <c r="D14" s="42" t="s">
+      <c r="D14" s="46" t="s">
         <v>11</v>
       </c>
-      <c r="E14" s="43"/>
+      <c r="E14" s="47"/>
       <c r="F14" s="16"/>
       <c r="G14" s="11"/>
       <c r="H14" s="14"/>
@@ -1614,8 +1967,8 @@
     </row>
     <row r="15" spans="3:13" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C15" s="4"/>
-      <c r="D15" s="40"/>
-      <c r="E15" s="41"/>
+      <c r="D15" s="38"/>
+      <c r="E15" s="40"/>
       <c r="F15" s="16"/>
       <c r="G15" s="11"/>
       <c r="H15" s="14"/>
@@ -1639,10 +1992,10 @@
     </row>
     <row r="17" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C17" s="4"/>
-      <c r="D17" s="42" t="s">
+      <c r="D17" s="46" t="s">
         <v>3</v>
       </c>
-      <c r="E17" s="43"/>
+      <c r="E17" s="47"/>
       <c r="F17" s="17"/>
       <c r="G17" s="11"/>
       <c r="H17" s="14"/>
@@ -1654,8 +2007,8 @@
     </row>
     <row r="18" spans="1:13" ht="107.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C18" s="4"/>
-      <c r="D18" s="40"/>
-      <c r="E18" s="41"/>
+      <c r="D18" s="38"/>
+      <c r="E18" s="40"/>
       <c r="F18" s="19"/>
       <c r="H18" s="14"/>
       <c r="I18" s="11"/>
@@ -1676,14 +2029,14 @@
     </row>
     <row r="20" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C20" s="4"/>
-      <c r="D20" s="42" t="s">
+      <c r="D20" s="46" t="s">
         <v>7</v>
       </c>
-      <c r="E20" s="43"/>
-      <c r="F20" s="46" t="s">
+      <c r="E20" s="47"/>
+      <c r="F20" s="41" t="s">
         <v>32</v>
       </c>
-      <c r="G20" s="47"/>
+      <c r="G20" s="43"/>
       <c r="H20" s="44" t="s">
         <v>1</v>
       </c>
@@ -1695,12 +2048,12 @@
     </row>
     <row r="21" spans="1:13" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C21" s="4"/>
-      <c r="D21" s="40"/>
-      <c r="E21" s="41"/>
-      <c r="F21" s="46"/>
-      <c r="G21" s="47"/>
-      <c r="H21" s="40"/>
-      <c r="I21" s="41"/>
+      <c r="D21" s="38"/>
+      <c r="E21" s="40"/>
+      <c r="F21" s="41"/>
+      <c r="G21" s="43"/>
+      <c r="H21" s="38"/>
+      <c r="I21" s="40"/>
       <c r="J21" s="16"/>
       <c r="K21" s="11"/>
       <c r="L21" s="14"/>
@@ -1718,10 +2071,10 @@
     </row>
     <row r="23" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C23" s="4"/>
-      <c r="D23" s="42" t="s">
+      <c r="D23" s="46" t="s">
         <v>10</v>
       </c>
-      <c r="E23" s="43"/>
+      <c r="E23" s="47"/>
       <c r="F23" s="8"/>
       <c r="G23" s="21"/>
       <c r="H23" s="21"/>
@@ -1735,16 +2088,16 @@
     </row>
     <row r="24" spans="1:13" ht="113.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C24" s="4"/>
-      <c r="D24" s="40"/>
-      <c r="E24" s="41"/>
+      <c r="D24" s="38"/>
+      <c r="E24" s="40"/>
       <c r="F24" s="5"/>
       <c r="G24" s="10"/>
       <c r="H24" s="10"/>
       <c r="I24" s="10"/>
       <c r="J24" s="6"/>
       <c r="K24" s="22"/>
-      <c r="L24" s="40"/>
-      <c r="M24" s="41"/>
+      <c r="L24" s="38"/>
+      <c r="M24" s="40"/>
     </row>
     <row r="25" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D25" s="12"/>
@@ -1771,8 +2124,8 @@
       <c r="A27" s="4"/>
       <c r="B27" s="5"/>
       <c r="C27" s="6"/>
-      <c r="D27" s="40"/>
-      <c r="E27" s="41"/>
+      <c r="D27" s="38"/>
+      <c r="E27" s="40"/>
       <c r="F27" s="11"/>
       <c r="J27" s="14"/>
       <c r="K27" s="11"/>
@@ -1795,10 +2148,10 @@
       </c>
       <c r="B29" s="45"/>
       <c r="C29" s="24"/>
-      <c r="D29" s="42" t="s">
+      <c r="D29" s="46" t="s">
         <v>15</v>
       </c>
-      <c r="E29" s="43"/>
+      <c r="E29" s="47"/>
       <c r="F29" s="8"/>
       <c r="G29" s="21"/>
       <c r="H29" s="21"/>
@@ -1809,11 +2162,11 @@
       <c r="M29" s="11"/>
     </row>
     <row r="30" spans="1:13" ht="322.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="40"/>
-      <c r="B30" s="41"/>
+      <c r="A30" s="38"/>
+      <c r="B30" s="40"/>
       <c r="C30" s="24"/>
-      <c r="D30" s="40"/>
-      <c r="E30" s="41"/>
+      <c r="D30" s="38"/>
+      <c r="E30" s="40"/>
       <c r="F30" s="19"/>
       <c r="G30" s="20"/>
       <c r="H30" s="20"/>
@@ -1831,44 +2184,44 @@
       <c r="M31" s="7"/>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A32" s="42" t="s">
+      <c r="A32" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="B32" s="43"/>
+      <c r="B32" s="47"/>
       <c r="C32" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="D32" s="42" t="s">
+      <c r="D32" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="E32" s="43"/>
-      <c r="F32" s="46" t="s">
+      <c r="E32" s="47"/>
+      <c r="F32" s="41" t="s">
         <v>31</v>
       </c>
-      <c r="G32" s="49"/>
-      <c r="H32" s="49"/>
-      <c r="I32" s="49"/>
-      <c r="J32" s="49"/>
-      <c r="K32" s="47"/>
-      <c r="L32" s="42" t="s">
+      <c r="G32" s="42"/>
+      <c r="H32" s="42"/>
+      <c r="I32" s="42"/>
+      <c r="J32" s="42"/>
+      <c r="K32" s="43"/>
+      <c r="L32" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="M32" s="43"/>
+      <c r="M32" s="47"/>
     </row>
     <row r="33" spans="1:13" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="50"/>
-      <c r="B33" s="48"/>
+      <c r="A33" s="48"/>
+      <c r="B33" s="39"/>
       <c r="C33" s="16"/>
-      <c r="D33" s="40"/>
-      <c r="E33" s="41"/>
-      <c r="F33" s="46"/>
-      <c r="G33" s="49"/>
-      <c r="H33" s="49"/>
-      <c r="I33" s="49"/>
-      <c r="J33" s="49"/>
-      <c r="K33" s="47"/>
-      <c r="L33" s="40"/>
-      <c r="M33" s="48"/>
+      <c r="D33" s="38"/>
+      <c r="E33" s="40"/>
+      <c r="F33" s="41"/>
+      <c r="G33" s="42"/>
+      <c r="H33" s="42"/>
+      <c r="I33" s="42"/>
+      <c r="J33" s="42"/>
+      <c r="K33" s="43"/>
+      <c r="L33" s="38"/>
+      <c r="M33" s="39"/>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A34" s="20"/>
@@ -1888,38 +2241,25 @@
     </row>
     <row r="36" spans="1:13" ht="213.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C36" s="4"/>
-      <c r="D36" s="40"/>
-      <c r="E36" s="41"/>
+      <c r="D36" s="38"/>
+      <c r="E36" s="40"/>
       <c r="F36" s="11"/>
     </row>
     <row r="38" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="E38" s="25"/>
       <c r="F38" s="25"/>
-      <c r="H38" s="40"/>
-      <c r="I38" s="48"/>
+      <c r="H38" s="38"/>
+      <c r="I38" s="39"/>
     </row>
     <row r="91" ht="0.75" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="41">
-    <mergeCell ref="H38:I38"/>
-    <mergeCell ref="D36:E36"/>
-    <mergeCell ref="F32:K32"/>
-    <mergeCell ref="A29:B29"/>
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="A30:B30"/>
-    <mergeCell ref="D30:E30"/>
-    <mergeCell ref="A33:B33"/>
-    <mergeCell ref="D33:E33"/>
-    <mergeCell ref="F33:K33"/>
-    <mergeCell ref="A32:B32"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="L23:M23"/>
-    <mergeCell ref="D24:E24"/>
-    <mergeCell ref="L24:M24"/>
-    <mergeCell ref="D26:E26"/>
-    <mergeCell ref="D35:E35"/>
-    <mergeCell ref="L32:M32"/>
-    <mergeCell ref="L33:M33"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="D8:E8"/>
     <mergeCell ref="H20:I20"/>
     <mergeCell ref="H21:I21"/>
     <mergeCell ref="H11:I11"/>
@@ -1936,12 +2276,25 @@
     <mergeCell ref="D12:E12"/>
     <mergeCell ref="D11:E11"/>
     <mergeCell ref="D23:E23"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="L23:M23"/>
+    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="L24:M24"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="D35:E35"/>
+    <mergeCell ref="L32:M32"/>
+    <mergeCell ref="L33:M33"/>
+    <mergeCell ref="H38:I38"/>
+    <mergeCell ref="D36:E36"/>
+    <mergeCell ref="F32:K32"/>
+    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="A30:B30"/>
+    <mergeCell ref="D30:E30"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="F33:K33"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="D32:E32"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>